<commit_message>
tabtools: modularize internals, add hrcomptab, drop fittab/hrtab; upd...
</commit_message>
<xml_diff>
--- a/msm/demo/msm_report.xlsx
+++ b/msm/demo/msm_report.xlsx
@@ -94,13 +94,13 @@
     <t>Variable</t>
   </si>
   <si>
-    <t>treatment</t>
-  </si>
-  <si>
-    <t>period</t>
-  </si>
-  <si>
-    <t>_msm_period_sq</t>
+    <t>Treatment</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Period^2</t>
   </si>
   <si>
     <t>age</t>
@@ -109,7 +109,7 @@
     <t>sex</t>
   </si>
   <si>
-    <t>_cons</t>
+    <t>Constant</t>
   </si>
   <si>
     <t>OR</t>
@@ -179,466 +179,493 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="268">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="274">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1477,7 +1504,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="208">
+  <borders count="214">
     <border>
       <left/>
       <right/>
@@ -2308,6 +2335,48 @@
     <border>
       <left style="none"/>
       <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
       <top style="thin"/>
       <bottom style="none"/>
       <diagonal style="none"/>
@@ -2890,7 +2959,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="208">
+  <cellXfs count="214">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -3220,238 +3289,238 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0"/>
-    <xf numFmtId="0" fontId="109" fillId="0" borderId="89" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="109" fillId="0" borderId="89" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="110" fillId="0" borderId="90" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="111" fillId="0" borderId="91" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="112" fillId="0" borderId="92" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="113" fillId="0" borderId="93" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="114" fillId="0" borderId="94" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="115" fillId="0" borderId="95" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="110" fillId="0" borderId="90" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="116" fillId="0" borderId="96" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="111" fillId="0" borderId="91" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="117" fillId="0" borderId="97" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="112" fillId="0" borderId="92" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="118" fillId="0" borderId="98" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="113" fillId="0" borderId="93" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="119" fillId="0" borderId="99" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="114" fillId="0" borderId="94" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="120" fillId="0" borderId="100" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="115" fillId="0" borderId="95" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="121" fillId="0" borderId="101" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="116" fillId="0" borderId="96" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="122" fillId="0" borderId="102" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="118" fillId="0" borderId="97" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="124" fillId="0" borderId="103" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="120" fillId="0" borderId="98" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="126" fillId="0" borderId="104" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="122" fillId="0" borderId="99" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="128" fillId="0" borderId="105" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="124" fillId="0" borderId="100" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="130" fillId="0" borderId="106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="125" fillId="0" borderId="101" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="131" fillId="0" borderId="107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="126" fillId="0" borderId="102" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="132" fillId="0" borderId="108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="127" fillId="0" borderId="103" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="133" fillId="0" borderId="109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="128" fillId="0" borderId="104" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="134" fillId="0" borderId="110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="129" fillId="0" borderId="105" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="135" fillId="0" borderId="111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="130" fillId="0" borderId="106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="136" fillId="0" borderId="112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="131" fillId="0" borderId="107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="137" fillId="0" borderId="113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="132" fillId="0" borderId="108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="138" fillId="0" borderId="114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="133" fillId="0" borderId="109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="139" fillId="0" borderId="115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="134" fillId="0" borderId="110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="140" fillId="0" borderId="116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="135" fillId="0" borderId="111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="141" fillId="0" borderId="117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="136" fillId="0" borderId="112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="142" fillId="0" borderId="118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="138" fillId="0" borderId="113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="144" fillId="0" borderId="119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="140" fillId="0" borderId="114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="146" fillId="0" borderId="120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="142" fillId="0" borderId="115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="148" fillId="0" borderId="121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="144" fillId="0" borderId="116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="150" fillId="0" borderId="122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="145" fillId="0" borderId="117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="151" fillId="0" borderId="123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="146" fillId="0" borderId="118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="152" fillId="0" borderId="124" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="147" fillId="0" borderId="119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="153" fillId="0" borderId="125" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="148" fillId="0" borderId="120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="154" fillId="0" borderId="126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="149" fillId="12" borderId="121" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="155" fillId="12" borderId="127" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="150" fillId="13" borderId="122" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="156" fillId="13" borderId="128" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="151" fillId="14" borderId="123" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="157" fillId="14" borderId="129" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="152" fillId="15" borderId="124" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="158" fillId="15" borderId="130" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="153" fillId="16" borderId="125" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="159" fillId="16" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="154" fillId="17" borderId="126" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="160" fillId="17" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="155" fillId="18" borderId="127" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="161" fillId="18" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="156" fillId="19" borderId="128" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="162" fillId="19" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="157" fillId="20" borderId="129" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="163" fillId="20" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="158" fillId="21" borderId="130" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="164" fillId="21" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="159" fillId="22" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="165" fillId="22" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="160" fillId="23" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="166" fillId="23" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="161" fillId="24" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="167" fillId="24" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="162" fillId="0" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="163" fillId="0" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="164" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="165" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="166" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="167" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="168" fillId="25" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="168" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="169" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="170" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="171" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="172" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="173" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="174" fillId="25" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="169" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="170" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="171" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="172" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="173" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="174" fillId="0" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="0" fontId="175" fillId="0" borderId="147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3469,30 +3538,30 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="179" fillId="0" borderId="151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="180" fillId="0" borderId="152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="181" fillId="0" borderId="153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="182" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="182" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="183" fillId="0" borderId="155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="184" fillId="0" borderId="156" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="185" fillId="0" borderId="157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="185" fillId="0" borderId="157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3500,7 +3569,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="187" fillId="0" borderId="159" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="187" fillId="0" borderId="159" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3508,7 +3577,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="189" fillId="0" borderId="161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="189" fillId="0" borderId="161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3516,32 +3585,32 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="191" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="191" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="192" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="193" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="194" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="195" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="196" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="197" fillId="0" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="192" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="193" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="194" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="195" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="196" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="197" fillId="26" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="198" fillId="0" borderId="170" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -3564,135 +3633,159 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="203" fillId="0" borderId="175" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="203" fillId="26" borderId="175" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="204" fillId="0" borderId="176" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="205" fillId="0" borderId="176" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="205" fillId="0" borderId="177" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="206" fillId="0" borderId="178" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="207" fillId="0" borderId="179" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="208" fillId="0" borderId="180" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="209" fillId="0" borderId="181" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="211" fillId="0" borderId="182" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="207" fillId="0" borderId="177" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="213" fillId="0" borderId="183" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="209" fillId="0" borderId="178" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="215" fillId="0" borderId="184" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="211" fillId="0" borderId="179" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="217" fillId="0" borderId="185" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="213" fillId="27" borderId="180" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="219" fillId="27" borderId="186" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="215" fillId="28" borderId="181" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="221" fillId="28" borderId="187" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="217" fillId="29" borderId="182" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="223" fillId="29" borderId="188" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="219" fillId="30" borderId="183" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="225" fillId="30" borderId="189" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="221" fillId="0" borderId="184" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="223" fillId="0" borderId="185" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="225" fillId="0" borderId="186" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="227" fillId="0" borderId="187" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="227" fillId="0" borderId="190" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="229" fillId="0" borderId="191" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="231" fillId="0" borderId="192" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="233" fillId="0" borderId="193" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="229" fillId="0" borderId="188" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="231" fillId="0" borderId="189" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="233" fillId="0" borderId="190" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="235" fillId="0" borderId="191" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="235" fillId="0" borderId="194" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="237" fillId="0" borderId="195" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="239" fillId="0" borderId="196" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="241" fillId="0" borderId="197" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="237" fillId="0" borderId="192" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="239" fillId="0" borderId="193" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="241" fillId="0" borderId="194" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="243" fillId="0" borderId="195" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="243" fillId="0" borderId="198" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="245" fillId="0" borderId="199" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="247" fillId="0" borderId="200" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="249" fillId="0" borderId="201" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="245" fillId="0" borderId="196" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="247" fillId="0" borderId="197" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="249" fillId="0" borderId="198" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="251" fillId="0" borderId="199" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="251" fillId="0" borderId="202" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="253" fillId="0" borderId="203" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="255" fillId="0" borderId="204" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="257" fillId="0" borderId="205" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="253" fillId="0" borderId="200" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="255" fillId="0" borderId="201" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="257" fillId="0" borderId="202" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="259" fillId="0" borderId="203" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="259" fillId="0" borderId="206" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="261" fillId="0" borderId="207" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="263" fillId="0" borderId="208" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="265" fillId="0" borderId="209" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="261" fillId="0" borderId="204" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="263" fillId="0" borderId="205" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="206" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="267" fillId="0" borderId="207" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="267" fillId="0" borderId="210" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="269" fillId="0" borderId="211" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="271" fillId="0" borderId="212" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="273" fillId="0" borderId="213" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3827,115 +3920,115 @@
   </cols>
   <sheetData>
     <row r="1" s="84" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="176" t="s">
+      <c r="A1" s="182" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="177" t="s">
+      <c r="B1" s="183" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="178" t="s">
+      <c r="C1" s="184" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="179" t="s">
+      <c r="D1" s="185" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="180" t="s">
+      <c r="A2" s="186" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="181" t="s">
+      <c r="B2" s="187" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="182" t="s">
+      <c r="C2" s="188" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="183" t="s">
+      <c r="D2" s="189" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="184" t="s">
+      <c r="A3" s="190" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="185">
-        <v>3</v>
-      </c>
-      <c r="C3" s="186">
-        <v>3</v>
-      </c>
-      <c r="D3" s="187">
-        <v>3</v>
+      <c r="B3" s="191">
+        <v>0.7672943522249035</v>
+      </c>
+      <c r="C3" s="192" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="193" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="188" t="s">
+      <c r="A4" s="194" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="189">
-        <v>4</v>
-      </c>
-      <c r="C4" s="190">
-        <v>4</v>
-      </c>
-      <c r="D4" s="191">
-        <v>4</v>
+      <c r="B4" s="195">
+        <v>0.96990480543369195</v>
+      </c>
+      <c r="C4" s="196" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="197" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="192" t="s">
+      <c r="A5" s="198" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="193">
-        <v>5</v>
-      </c>
-      <c r="C5" s="194">
-        <v>5</v>
-      </c>
-      <c r="D5" s="195">
-        <v>5</v>
+      <c r="B5" s="199">
+        <v>1.0135738905506451</v>
+      </c>
+      <c r="C5" s="200" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="201" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="196" t="s">
+      <c r="A6" s="202" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="197">
-        <v>6</v>
-      </c>
-      <c r="C6" s="198">
-        <v>6</v>
-      </c>
-      <c r="D6" s="199">
-        <v>6</v>
+      <c r="B6" s="203">
+        <v>1.052812145678234</v>
+      </c>
+      <c r="C6" s="204" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="205" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="200" t="s">
+      <c r="A7" s="206" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="201">
-        <v>7</v>
-      </c>
-      <c r="C7" s="202">
-        <v>7</v>
-      </c>
-      <c r="D7" s="203">
-        <v>7</v>
+      <c r="B7" s="207">
+        <v>0.91156457885765974</v>
+      </c>
+      <c r="C7" s="208" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="209" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="204" t="s">
+      <c r="A8" s="210" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="205">
-        <v>8</v>
-      </c>
-      <c r="C8" s="206">
-        <v>8</v>
-      </c>
-      <c r="D8" s="207">
-        <v>8</v>
+      <c r="B8" s="211">
+        <v>0.00049674249516860002</v>
+      </c>
+      <c r="C8" s="212" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="213" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>